<commit_message>
[COMPARISON]: Add Encryption mode
</commit_message>
<xml_diff>
--- a/jour_4/Comparatif cloud.xlsx
+++ b/jour_4/Comparatif cloud.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trist\Documents\Ecole\M2\data-cloud\exercise-data-cloud\jour_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8349096-76A7-40F6-A5CE-3887A898641E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CE5DBC-8F64-4335-A5F2-F1FB41C0ECFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{79880B3A-6D65-41F7-B4B7-054A8164B96A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>Critère</t>
   </si>
@@ -141,6 +141,113 @@
   </si>
   <si>
     <t>Moins de services avancés, moins d’exemples/tutos en ligne</t>
+  </si>
+  <si>
+    <t>Mode de chiffrement</t>
+  </si>
+  <si>
+    <r>
+      <t>At rest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : AES-256, choix entre SSE-S3, SSE-KMS, BYOK </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>In transit : TLS 1.2+ obligatoire</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>At rest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : AES-256, Azure Key Vault, BYOK possible</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In transit : TLS 1.2+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>At rest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : AES-256, Cloud KMS, BYOK possible</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In transit : TLS 1.2+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>At rest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : AES-256, Customer Key Manager (CKM), BYOK possible </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>In transit : TLS 1.2+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -205,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,6 +321,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -550,11 +663,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53271ADF-7726-4643-961A-CED310EB0958}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.6640625" customWidth="1"/>
     <col min="3" max="3" width="52.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="51.5546875" bestFit="1" customWidth="1"/>
@@ -679,7 +792,37 @@
         <v>34</v>
       </c>
     </row>
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="4"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>